<commit_message>
data(gis): publish GeoLibre analysis yilan-public-facility-hazard-exposure-2026-09-26-update
</commit_message>
<xml_diff>
--- a/GeoLibre-Web/analysis/yilan-public-facility-hazard-exposure-2026-09-26-update/result.xlsx
+++ b/GeoLibre-Web/analysis/yilan-public-facility-hazard-exposure-2026-09-26-update/result.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分析結果" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="統計摘要" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分析參數" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="資料來源" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全部291處設施" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="分析結果" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="統計摘要" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="分析參數" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="資料來源" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="全部291處設施" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'分析結果'!$A$1:$T$172</definedName>
@@ -27,16 +27,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -47,7 +44,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -55,21 +52,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -461,102 +449,102 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>設施編號</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>設施名稱</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>設施類型</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>資料來源</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>經度</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>緯度</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>source_month</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>點位說明</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>TWD97東向座標</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>TWD97北向座標</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>image_pixel_x</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>image_pixel_y</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>圖面覆蓋狀態</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>新版圖面分類</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>影像判讀狀態</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>距最近中高潛勢圖色_公尺</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>最近中高潛勢級別</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>300公尺內中高潛勢候選</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>篩選說明</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>sampled_rgb_class_pixels_5x5</t>
         </is>
@@ -14605,17 +14593,17 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>統計項目</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>數量</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>說明</t>
         </is>
@@ -14776,12 +14764,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>參數</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>設定</t>
         </is>
@@ -14896,37 +14884,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>圖層／資料</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>提供單位</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>來源網址</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>資料版次／期間</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>取得日期</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>分析用途</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>限制</t>
         </is>
@@ -15303,102 +15291,102 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>設施編號</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>設施名稱</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>設施類型</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>資料來源</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>經度</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>緯度</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>source_month</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>點位說明</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>TWD97東向座標</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>TWD97北向座標</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>image_pixel_x</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>image_pixel_y</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>圖面覆蓋狀態</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>新版圖面分類</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>影像判讀狀態</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>距最近中高潛勢圖色_公尺</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>最近中高潛勢級別</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>300公尺內中高潛勢候選</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>篩選說明</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>sampled_rgb_class_pixels_5x5</t>
         </is>

</xml_diff>